<commit_message>
Resultados de análisis problema2 (1M iteraciones)
</commit_message>
<xml_diff>
--- a/Nuevos DeepWins/Problem2_Checkerboard6x6/Res/Comparativa_12_Neuronas.xlsx
+++ b/Nuevos DeepWins/Problem2_Checkerboard6x6/Res/Comparativa_12_Neuronas.xlsx
@@ -581,35 +581,43 @@
         <v>0.1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.24992</v>
+        <v>0.213166</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1790730194</v>
+        <v>1790730142</v>
       </c>
       <c r="E2" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F2" t="n">
         <v>200000</v>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>0.654096</v>
+      </c>
       <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="inlineStr"/>
+        <v>0.6343</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.644046</v>
+      </c>
       <c r="J2" t="n">
-        <v>0.249813</v>
-      </c>
-      <c r="K2" t="inlineStr"/>
+        <v>0.214602</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.62963</v>
+      </c>
       <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="inlineStr"/>
+        <v>0.636364</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.632979</v>
+      </c>
       <c r="N2" t="n">
         <v>0.2</v>
       </c>
@@ -644,23 +652,23 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_10.txt</t>
+          <t>_2_12_1_1790730142_6.txt</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z2" t="n">
         <v>12</v>
       </c>
       <c r="AA2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -674,7 +682,7 @@
         <v>0.1</v>
       </c>
       <c r="B3" t="n">
-        <v>0.249874</v>
+        <v>0.249984</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -690,27 +698,19 @@
       <c r="F3" t="n">
         <v>200000</v>
       </c>
-      <c r="G3" t="n">
-        <v>0.663043</v>
-      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>0.07692300000000001</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.137853</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
-        <v>0.24988</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.6</v>
-      </c>
+        <v>0.249737</v>
+      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
-        <v>0.048128</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.08910899999999999</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
         <v>0.2</v>
       </c>
@@ -745,7 +745,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_8.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_7.txt</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -775,7 +775,7 @@
         <v>0.1</v>
       </c>
       <c r="B4" t="n">
-        <v>0.209851</v>
+        <v>0.222749</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -792,25 +792,25 @@
         <v>200000</v>
       </c>
       <c r="G4" t="n">
-        <v>0.670833</v>
+        <v>0.574932</v>
       </c>
       <c r="H4" t="n">
-        <v>0.609079</v>
+        <v>0.532156</v>
       </c>
       <c r="I4" t="n">
-        <v>0.638467</v>
+        <v>0.552718</v>
       </c>
       <c r="J4" t="n">
-        <v>0.208664</v>
+        <v>0.226198</v>
       </c>
       <c r="K4" t="n">
-        <v>0.641176</v>
+        <v>0.556818</v>
       </c>
       <c r="L4" t="n">
-        <v>0.582888</v>
+        <v>0.524064</v>
       </c>
       <c r="M4" t="n">
-        <v>0.610644</v>
+        <v>0.539945</v>
       </c>
       <c r="N4" t="n">
         <v>0.2</v>
@@ -846,7 +846,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_10.txt</t>
+          <t>_2_12_1_1790730142_16.txt</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -876,7 +876,7 @@
         <v>0.1</v>
       </c>
       <c r="B5" t="n">
-        <v>0.249907</v>
+        <v>0.249935</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
-        <v>0.249831</v>
+        <v>0.249791</v>
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
@@ -939,7 +939,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_18.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_6.txt</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -969,7 +969,7 @@
         <v>0.1</v>
       </c>
       <c r="B6" t="n">
-        <v>0.213282</v>
+        <v>0.209851</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -986,25 +986,25 @@
         <v>200000</v>
       </c>
       <c r="G6" t="n">
-        <v>0.642595</v>
+        <v>0.670833</v>
       </c>
       <c r="H6" t="n">
-        <v>0.662043</v>
+        <v>0.609079</v>
       </c>
       <c r="I6" t="n">
-        <v>0.652174</v>
+        <v>0.638467</v>
       </c>
       <c r="J6" t="n">
-        <v>0.215239</v>
+        <v>0.208664</v>
       </c>
       <c r="K6" t="n">
-        <v>0.6376810000000001</v>
+        <v>0.641176</v>
       </c>
       <c r="L6" t="n">
-        <v>0.705882</v>
+        <v>0.582888</v>
       </c>
       <c r="M6" t="n">
-        <v>0.670051</v>
+        <v>0.610644</v>
       </c>
       <c r="N6" t="n">
         <v>0.2</v>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_1.txt</t>
+          <t>_2_12_1_1790730142_10.txt</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -1070,7 +1070,7 @@
         <v>0.1</v>
       </c>
       <c r="B7" t="n">
-        <v>0.249973</v>
+        <v>0.249401</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1086,19 +1086,27 @@
       <c r="F7" t="n">
         <v>200000</v>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>0.5293330000000001</v>
+      </c>
       <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="inlineStr"/>
+        <v>0.50063</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.514582</v>
+      </c>
       <c r="J7" t="n">
-        <v>0.249742</v>
-      </c>
-      <c r="K7" t="inlineStr"/>
+        <v>0.251069</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.445596</v>
+      </c>
       <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="inlineStr"/>
+        <v>0.459893</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.452632</v>
+      </c>
       <c r="N7" t="n">
         <v>0.2</v>
       </c>
@@ -1133,7 +1141,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_12.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_13.txt</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
@@ -1163,43 +1171,35 @@
         <v>0.1</v>
       </c>
       <c r="B8" t="n">
-        <v>0.210905</v>
+        <v>0.249879</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1790730142</v>
+        <v>1790730194</v>
       </c>
       <c r="E8" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F8" t="n">
         <v>200000</v>
       </c>
-      <c r="G8" t="n">
-        <v>0.652288</v>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>0.629256</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.6405650000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="n">
-        <v>0.210832</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0.637838</v>
-      </c>
+        <v>0.249846</v>
+      </c>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
-        <v>0.631016</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.634409</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
         <v>0.2</v>
       </c>
@@ -1234,23 +1234,23 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_18.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_15.txt</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z8" t="n">
         <v>12</v>
       </c>
       <c r="AA8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
@@ -1264,42 +1264,42 @@
         <v>0.1</v>
       </c>
       <c r="B9" t="n">
-        <v>0.222749</v>
+        <v>0.249874</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1790730142</v>
+        <v>1790730194</v>
       </c>
       <c r="E9" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F9" t="n">
         <v>200000</v>
       </c>
       <c r="G9" t="n">
-        <v>0.574932</v>
+        <v>0.663043</v>
       </c>
       <c r="H9" t="n">
-        <v>0.532156</v>
+        <v>0.07692300000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>0.552718</v>
+        <v>0.137853</v>
       </c>
       <c r="J9" t="n">
-        <v>0.226198</v>
+        <v>0.24988</v>
       </c>
       <c r="K9" t="n">
-        <v>0.556818</v>
+        <v>0.6</v>
       </c>
       <c r="L9" t="n">
-        <v>0.524064</v>
+        <v>0.048128</v>
       </c>
       <c r="M9" t="n">
-        <v>0.539945</v>
+        <v>0.08910899999999999</v>
       </c>
       <c r="N9" t="n">
         <v>0.2</v>
@@ -1335,23 +1335,23 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_16.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_8.txt</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z9" t="n">
         <v>12</v>
       </c>
       <c r="AA9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
@@ -1365,35 +1365,43 @@
         <v>0.1</v>
       </c>
       <c r="B10" t="n">
-        <v>0.249981</v>
+        <v>0.222045</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1790730194</v>
+        <v>1790730142</v>
       </c>
       <c r="E10" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F10" t="n">
         <v>200000</v>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>0.594796</v>
+      </c>
       <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="inlineStr"/>
+        <v>0.6052959999999999</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.6</v>
+      </c>
       <c r="J10" t="n">
-        <v>0.249734</v>
-      </c>
-      <c r="K10" t="inlineStr"/>
+        <v>0.222816</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.581152</v>
+      </c>
       <c r="L10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" t="inlineStr"/>
+        <v>0.593583</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.587302</v>
+      </c>
       <c r="N10" t="n">
         <v>0.2</v>
       </c>
@@ -1428,23 +1436,23 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_17.txt</t>
+          <t>_2_12_1_1790730142_14.txt</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z10" t="n">
         <v>12</v>
       </c>
       <c r="AA10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
@@ -1458,7 +1466,7 @@
         <v>0.1</v>
       </c>
       <c r="B11" t="n">
-        <v>0.249969</v>
+        <v>0.249981</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1480,7 +1488,7 @@
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="n">
-        <v>0.249749</v>
+        <v>0.249734</v>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
@@ -1521,7 +1529,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_3.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_17.txt</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
@@ -1551,7 +1559,7 @@
         <v>0.1</v>
       </c>
       <c r="B12" t="n">
-        <v>0.222952</v>
+        <v>0.220684</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1568,25 +1576,25 @@
         <v>200000</v>
       </c>
       <c r="G12" t="n">
-        <v>0.617574</v>
+        <v>0.590909</v>
       </c>
       <c r="H12" t="n">
-        <v>0.629256</v>
+        <v>0.622951</v>
       </c>
       <c r="I12" t="n">
-        <v>0.62336</v>
+        <v>0.606507</v>
       </c>
       <c r="J12" t="n">
-        <v>0.223623</v>
+        <v>0.221005</v>
       </c>
       <c r="K12" t="n">
-        <v>0.591133</v>
+        <v>0.582915</v>
       </c>
       <c r="L12" t="n">
-        <v>0.641711</v>
+        <v>0.620321</v>
       </c>
       <c r="M12" t="n">
-        <v>0.615385</v>
+        <v>0.601036</v>
       </c>
       <c r="N12" t="n">
         <v>0.2</v>
@@ -1622,7 +1630,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_12.txt</t>
+          <t>_2_12_1_1790730142_8.txt</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
@@ -1652,7 +1660,7 @@
         <v>0.1</v>
       </c>
       <c r="B13" t="n">
-        <v>0.215142</v>
+        <v>0.218388</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1669,25 +1677,25 @@
         <v>200000</v>
       </c>
       <c r="G13" t="n">
-        <v>0.6676260000000001</v>
+        <v>0.623529</v>
       </c>
       <c r="H13" t="n">
-        <v>0.58512</v>
+        <v>0.6683480000000001</v>
       </c>
       <c r="I13" t="n">
-        <v>0.623656</v>
+        <v>0.645161</v>
       </c>
       <c r="J13" t="n">
-        <v>0.215538</v>
+        <v>0.222459</v>
       </c>
       <c r="K13" t="n">
-        <v>0.65896</v>
+        <v>0.558824</v>
       </c>
       <c r="L13" t="n">
         <v>0.609626</v>
       </c>
       <c r="M13" t="n">
-        <v>0.633333</v>
+        <v>0.58312</v>
       </c>
       <c r="N13" t="n">
         <v>0.2</v>
@@ -1723,7 +1731,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_4.txt</t>
+          <t>_2_12_1_1790730142_13.txt</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
@@ -1753,7 +1761,7 @@
         <v>0.1</v>
       </c>
       <c r="B14" t="n">
-        <v>0.225402</v>
+        <v>0.215814</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1770,25 +1778,25 @@
         <v>200000</v>
       </c>
       <c r="G14" t="n">
-        <v>0.59611</v>
+        <v>0.635251</v>
       </c>
       <c r="H14" t="n">
-        <v>0.656999</v>
+        <v>0.654477</v>
       </c>
       <c r="I14" t="n">
-        <v>0.625075</v>
+        <v>0.64472</v>
       </c>
       <c r="J14" t="n">
-        <v>0.228309</v>
+        <v>0.217291</v>
       </c>
       <c r="K14" t="n">
-        <v>0.552885</v>
+        <v>0.6282720000000001</v>
       </c>
       <c r="L14" t="n">
-        <v>0.614973</v>
+        <v>0.641711</v>
       </c>
       <c r="M14" t="n">
-        <v>0.582278</v>
+        <v>0.634921</v>
       </c>
       <c r="N14" t="n">
         <v>0.2</v>
@@ -1824,7 +1832,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_19.txt</t>
+          <t>_2_12_1_1790730142_11.txt</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
@@ -1854,35 +1862,43 @@
         <v>0.1</v>
       </c>
       <c r="B15" t="n">
-        <v>0.249942</v>
+        <v>0.209168</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1790730194</v>
+        <v>1790730142</v>
       </c>
       <c r="E15" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F15" t="n">
         <v>200000</v>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="n">
+        <v>0.649235</v>
+      </c>
       <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="inlineStr"/>
+        <v>0.641866</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.64553</v>
+      </c>
       <c r="J15" t="n">
-        <v>0.249777</v>
-      </c>
-      <c r="K15" t="inlineStr"/>
+        <v>0.210112</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.6284149999999999</v>
+      </c>
       <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="inlineStr"/>
+        <v>0.614973</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.621622</v>
+      </c>
       <c r="N15" t="n">
         <v>0.2</v>
       </c>
@@ -1917,23 +1933,23 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_1.txt</t>
+          <t>_2_12_1_1790730142_7.txt</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z15" t="n">
         <v>12</v>
       </c>
       <c r="AA15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
@@ -1947,43 +1963,35 @@
         <v>0.1</v>
       </c>
       <c r="B16" t="n">
-        <v>0.213166</v>
+        <v>0.24998</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1790730142</v>
+        <v>1790730194</v>
       </c>
       <c r="E16" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F16" t="n">
         <v>200000</v>
       </c>
-      <c r="G16" t="n">
-        <v>0.654096</v>
-      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>0.6343</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0.644046</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="n">
-        <v>0.214602</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0.62963</v>
-      </c>
+        <v>0.249735</v>
+      </c>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="n">
-        <v>0.636364</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0.632979</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
         <v>0.2</v>
       </c>
@@ -2018,23 +2026,23 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_6.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_11.txt</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z16" t="n">
         <v>12</v>
       </c>
       <c r="AA16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
@@ -2048,35 +2056,43 @@
         <v>0.1</v>
       </c>
       <c r="B17" t="n">
-        <v>0.249984</v>
+        <v>0.222712</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1790730194</v>
+        <v>1790730142</v>
       </c>
       <c r="E17" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F17" t="n">
         <v>200000</v>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="n">
+        <v>0.5936709999999999</v>
+      </c>
       <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="inlineStr"/>
+        <v>0.591425</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.592546</v>
+      </c>
       <c r="J17" t="n">
-        <v>0.249737</v>
-      </c>
-      <c r="K17" t="inlineStr"/>
+        <v>0.224653</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.574468</v>
+      </c>
       <c r="L17" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" t="inlineStr"/>
+        <v>0.5775400000000001</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.576</v>
+      </c>
       <c r="N17" t="n">
         <v>0.2</v>
       </c>
@@ -2111,23 +2127,23 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_7.txt</t>
+          <t>_2_12_1_1790730142_17.txt</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z17" t="n">
         <v>12</v>
       </c>
       <c r="AA17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
@@ -2141,7 +2157,7 @@
         <v>0.1</v>
       </c>
       <c r="B18" t="n">
-        <v>0.24932</v>
+        <v>0.249977</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2157,27 +2173,19 @@
       <c r="F18" t="n">
         <v>200000</v>
       </c>
-      <c r="G18" t="n">
-        <v>0.5211440000000001</v>
-      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>0.528373</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0.524734</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="n">
-        <v>0.251792</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0.42381</v>
-      </c>
+        <v>0.249738</v>
+      </c>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
-        <v>0.475936</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0.448363</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="n">
         <v>0.2</v>
       </c>
@@ -2212,7 +2220,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_0.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_14.txt</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
@@ -2242,35 +2250,43 @@
         <v>0.1</v>
       </c>
       <c r="B19" t="n">
-        <v>0.249879</v>
+        <v>0.210905</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1790730194</v>
+        <v>1790730142</v>
       </c>
       <c r="E19" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F19" t="n">
         <v>200000</v>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="n">
+        <v>0.652288</v>
+      </c>
       <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" t="inlineStr"/>
+        <v>0.629256</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.6405650000000001</v>
+      </c>
       <c r="J19" t="n">
-        <v>0.249846</v>
-      </c>
-      <c r="K19" t="inlineStr"/>
+        <v>0.210832</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.637838</v>
+      </c>
       <c r="L19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" t="inlineStr"/>
+        <v>0.631016</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.634409</v>
+      </c>
       <c r="N19" t="n">
         <v>0.2</v>
       </c>
@@ -2305,23 +2321,23 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_15.txt</t>
+          <t>_2_12_1_1790730142_18.txt</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z19" t="n">
         <v>12</v>
       </c>
       <c r="AA19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC19" t="inlineStr">
@@ -2436,42 +2452,42 @@
         <v>0.1</v>
       </c>
       <c r="B21" t="n">
-        <v>0.249401</v>
+        <v>0.211887</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1790730194</v>
+        <v>1790730142</v>
       </c>
       <c r="E21" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F21" t="n">
         <v>200000</v>
       </c>
       <c r="G21" t="n">
-        <v>0.5293330000000001</v>
+        <v>0.654289</v>
       </c>
       <c r="H21" t="n">
-        <v>0.50063</v>
+        <v>0.644388</v>
       </c>
       <c r="I21" t="n">
-        <v>0.514582</v>
+        <v>0.649301</v>
       </c>
       <c r="J21" t="n">
-        <v>0.251069</v>
+        <v>0.213922</v>
       </c>
       <c r="K21" t="n">
-        <v>0.445596</v>
+        <v>0.644809</v>
       </c>
       <c r="L21" t="n">
-        <v>0.459893</v>
+        <v>0.631016</v>
       </c>
       <c r="M21" t="n">
-        <v>0.452632</v>
+        <v>0.637838</v>
       </c>
       <c r="N21" t="n">
         <v>0.2</v>
@@ -2507,23 +2523,23 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_13.txt</t>
+          <t>_2_12_1_1790730142_15.txt</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z21" t="n">
         <v>12</v>
       </c>
       <c r="AA21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC21" t="inlineStr">
@@ -2638,7 +2654,7 @@
         <v>0.1</v>
       </c>
       <c r="B23" t="n">
-        <v>0.249928</v>
+        <v>0.24936</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2655,25 +2671,25 @@
         <v>200000</v>
       </c>
       <c r="G23" t="n">
-        <v>0.537815</v>
+        <v>0.531044</v>
       </c>
       <c r="H23" t="n">
-        <v>0.080706</v>
+        <v>0.5069360000000001</v>
       </c>
       <c r="I23" t="n">
-        <v>0.140351</v>
+        <v>0.51871</v>
       </c>
       <c r="J23" t="n">
-        <v>0.249862</v>
+        <v>0.251423</v>
       </c>
       <c r="K23" t="n">
-        <v>0.391304</v>
+        <v>0.441026</v>
       </c>
       <c r="L23" t="n">
-        <v>0.048128</v>
+        <v>0.459893</v>
       </c>
       <c r="M23" t="n">
-        <v>0.085714</v>
+        <v>0.450262</v>
       </c>
       <c r="N23" t="n">
         <v>0.2</v>
@@ -2709,7 +2725,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_16.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_2.txt</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
@@ -2739,7 +2755,7 @@
         <v>0.1</v>
       </c>
       <c r="B24" t="n">
-        <v>0.249977</v>
+        <v>0.249509</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2755,19 +2771,27 @@
       <c r="F24" t="n">
         <v>200000</v>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="n">
+        <v>0.520567</v>
+      </c>
       <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="inlineStr"/>
+        <v>0.462799</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.489987</v>
+      </c>
       <c r="J24" t="n">
-        <v>0.249738</v>
-      </c>
-      <c r="K24" t="inlineStr"/>
+        <v>0.250785</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0.446237</v>
+      </c>
       <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="inlineStr"/>
+        <v>0.44385</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0.44504</v>
+      </c>
       <c r="N24" t="n">
         <v>0.2</v>
       </c>
@@ -2802,7 +2826,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_14.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_9.txt</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
@@ -2832,43 +2856,35 @@
         <v>0.1</v>
       </c>
       <c r="B25" t="n">
-        <v>0.222045</v>
+        <v>0.24992</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>1790730142</v>
+        <v>1790730194</v>
       </c>
       <c r="E25" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F25" t="n">
         <v>200000</v>
       </c>
-      <c r="G25" t="n">
-        <v>0.594796</v>
-      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>0.6052959999999999</v>
-      </c>
-      <c r="I25" t="n">
-        <v>0.6</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="n">
-        <v>0.222816</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0.581152</v>
-      </c>
+        <v>0.249813</v>
+      </c>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="n">
-        <v>0.593583</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0.587302</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M25" t="inlineStr"/>
       <c r="N25" t="n">
         <v>0.2</v>
       </c>
@@ -2903,23 +2919,23 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_14.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_10.txt</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z25" t="n">
         <v>12</v>
       </c>
       <c r="AA25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC25" t="inlineStr">
@@ -2933,7 +2949,7 @@
         <v>0.1</v>
       </c>
       <c r="B26" t="n">
-        <v>0.249935</v>
+        <v>0.249928</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2949,19 +2965,27 @@
       <c r="F26" t="n">
         <v>200000</v>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="n">
+        <v>0.537815</v>
+      </c>
       <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" t="inlineStr"/>
+        <v>0.080706</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.140351</v>
+      </c>
       <c r="J26" t="n">
-        <v>0.249791</v>
-      </c>
-      <c r="K26" t="inlineStr"/>
+        <v>0.249862</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0.391304</v>
+      </c>
       <c r="L26" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" t="inlineStr"/>
+        <v>0.048128</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0.085714</v>
+      </c>
       <c r="N26" t="n">
         <v>0.2</v>
       </c>
@@ -2996,7 +3020,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_6.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_16.txt</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
@@ -3026,35 +3050,43 @@
         <v>0.1</v>
       </c>
       <c r="B27" t="n">
-        <v>0.24998</v>
+        <v>0.213282</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1790730194</v>
+        <v>1790730142</v>
       </c>
       <c r="E27" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F27" t="n">
         <v>200000</v>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="n">
+        <v>0.642595</v>
+      </c>
       <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" t="inlineStr"/>
+        <v>0.662043</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.652174</v>
+      </c>
       <c r="J27" t="n">
-        <v>0.249735</v>
-      </c>
-      <c r="K27" t="inlineStr"/>
+        <v>0.215239</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0.6376810000000001</v>
+      </c>
       <c r="L27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" t="inlineStr"/>
+        <v>0.705882</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0.670051</v>
+      </c>
       <c r="N27" t="n">
         <v>0.2</v>
       </c>
@@ -3089,23 +3121,23 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_11.txt</t>
+          <t>_2_12_1_1790730142_1.txt</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z27" t="n">
         <v>12</v>
       </c>
       <c r="AA27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC27" t="inlineStr">
@@ -3119,42 +3151,42 @@
         <v>0.1</v>
       </c>
       <c r="B28" t="n">
-        <v>0.222712</v>
+        <v>0.249751</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1790730142</v>
+        <v>1790730194</v>
       </c>
       <c r="E28" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F28" t="n">
         <v>200000</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5936709999999999</v>
+        <v>0.513726</v>
       </c>
       <c r="H28" t="n">
-        <v>0.591425</v>
+        <v>0.330391</v>
       </c>
       <c r="I28" t="n">
-        <v>0.592546</v>
+        <v>0.402149</v>
       </c>
       <c r="J28" t="n">
-        <v>0.224653</v>
+        <v>0.250068</v>
       </c>
       <c r="K28" t="n">
-        <v>0.574468</v>
+        <v>0.457746</v>
       </c>
       <c r="L28" t="n">
-        <v>0.5775400000000001</v>
+        <v>0.347594</v>
       </c>
       <c r="M28" t="n">
-        <v>0.576</v>
+        <v>0.395137</v>
       </c>
       <c r="N28" t="n">
         <v>0.2</v>
@@ -3190,23 +3222,23 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_17.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_5.txt</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z28" t="n">
         <v>12</v>
       </c>
       <c r="AA28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC28" t="inlineStr">
@@ -3220,7 +3252,7 @@
         <v>0.1</v>
       </c>
       <c r="B29" t="n">
-        <v>0.209168</v>
+        <v>0.222952</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3237,25 +3269,25 @@
         <v>200000</v>
       </c>
       <c r="G29" t="n">
-        <v>0.649235</v>
+        <v>0.617574</v>
       </c>
       <c r="H29" t="n">
-        <v>0.641866</v>
+        <v>0.629256</v>
       </c>
       <c r="I29" t="n">
-        <v>0.64553</v>
+        <v>0.62336</v>
       </c>
       <c r="J29" t="n">
-        <v>0.210112</v>
+        <v>0.223623</v>
       </c>
       <c r="K29" t="n">
-        <v>0.6284149999999999</v>
+        <v>0.591133</v>
       </c>
       <c r="L29" t="n">
-        <v>0.614973</v>
+        <v>0.641711</v>
       </c>
       <c r="M29" t="n">
-        <v>0.621622</v>
+        <v>0.615385</v>
       </c>
       <c r="N29" t="n">
         <v>0.2</v>
@@ -3291,7 +3323,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_7.txt</t>
+          <t>_2_12_1_1790730142_12.txt</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
@@ -3321,42 +3353,42 @@
         <v>0.1</v>
       </c>
       <c r="B30" t="n">
-        <v>0.22163</v>
+        <v>0.24932</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1790730142</v>
+        <v>1790730194</v>
       </c>
       <c r="E30" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F30" t="n">
         <v>200000</v>
       </c>
       <c r="G30" t="n">
-        <v>0.612943</v>
+        <v>0.5211440000000001</v>
       </c>
       <c r="H30" t="n">
-        <v>0.633039</v>
+        <v>0.528373</v>
       </c>
       <c r="I30" t="n">
-        <v>0.622829</v>
+        <v>0.524734</v>
       </c>
       <c r="J30" t="n">
-        <v>0.224606</v>
+        <v>0.251792</v>
       </c>
       <c r="K30" t="n">
-        <v>0.596939</v>
+        <v>0.42381</v>
       </c>
       <c r="L30" t="n">
-        <v>0.625668</v>
+        <v>0.475936</v>
       </c>
       <c r="M30" t="n">
-        <v>0.610966</v>
+        <v>0.448363</v>
       </c>
       <c r="N30" t="n">
         <v>0.2</v>
@@ -3392,23 +3424,23 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_9.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_0.txt</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z30" t="n">
         <v>12</v>
       </c>
       <c r="AA30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC30" t="inlineStr">
@@ -3422,7 +3454,7 @@
         <v>0.1</v>
       </c>
       <c r="B31" t="n">
-        <v>0.24936</v>
+        <v>0.249969</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3438,27 +3470,19 @@
       <c r="F31" t="n">
         <v>200000</v>
       </c>
-      <c r="G31" t="n">
-        <v>0.531044</v>
-      </c>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>0.5069360000000001</v>
-      </c>
-      <c r="I31" t="n">
-        <v>0.51871</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="n">
-        <v>0.251423</v>
-      </c>
-      <c r="K31" t="n">
-        <v>0.441026</v>
-      </c>
+        <v>0.249749</v>
+      </c>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="n">
-        <v>0.459893</v>
-      </c>
-      <c r="M31" t="n">
-        <v>0.450262</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M31" t="inlineStr"/>
       <c r="N31" t="n">
         <v>0.2</v>
       </c>
@@ -3493,7 +3517,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_2.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_3.txt</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
@@ -3523,43 +3547,35 @@
         <v>0.1</v>
       </c>
       <c r="B32" t="n">
-        <v>0.218388</v>
+        <v>0.249962</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1790730142</v>
+        <v>1790730194</v>
       </c>
       <c r="E32" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F32" t="n">
         <v>200000</v>
       </c>
-      <c r="G32" t="n">
-        <v>0.623529</v>
-      </c>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>0.6683480000000001</v>
-      </c>
-      <c r="I32" t="n">
-        <v>0.645161</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr"/>
       <c r="J32" t="n">
-        <v>0.222459</v>
-      </c>
-      <c r="K32" t="n">
-        <v>0.558824</v>
-      </c>
+        <v>0.249766</v>
+      </c>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="n">
-        <v>0.609626</v>
-      </c>
-      <c r="M32" t="n">
-        <v>0.58312</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M32" t="inlineStr"/>
       <c r="N32" t="n">
         <v>0.2</v>
       </c>
@@ -3594,23 +3610,23 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_13.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_4.txt</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z32" t="n">
         <v>12</v>
       </c>
       <c r="AA32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC32" t="inlineStr">
@@ -3624,35 +3640,43 @@
         <v>0.1</v>
       </c>
       <c r="B33" t="n">
-        <v>0.249927</v>
+        <v>0.22534</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1790730194</v>
+        <v>1790730142</v>
       </c>
       <c r="E33" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F33" t="n">
         <v>200000</v>
       </c>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" t="n">
+        <v>0.642265</v>
+      </c>
       <c r="H33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" t="inlineStr"/>
+        <v>0.586381</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.613052</v>
+      </c>
       <c r="J33" t="n">
-        <v>0.249811</v>
-      </c>
-      <c r="K33" t="inlineStr"/>
+        <v>0.235937</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.559006</v>
+      </c>
       <c r="L33" t="n">
-        <v>0</v>
-      </c>
-      <c r="M33" t="inlineStr"/>
+        <v>0.481283</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0.517241</v>
+      </c>
       <c r="N33" t="n">
         <v>0.2</v>
       </c>
@@ -3687,23 +3711,23 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_19.txt</t>
+          <t>_2_12_1_1790730142_0.txt</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z33" t="n">
         <v>12</v>
       </c>
       <c r="AA33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC33" t="inlineStr">
@@ -3717,7 +3741,7 @@
         <v>0.1</v>
       </c>
       <c r="B34" t="n">
-        <v>0.249751</v>
+        <v>0.249927</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -3733,27 +3757,19 @@
       <c r="F34" t="n">
         <v>200000</v>
       </c>
-      <c r="G34" t="n">
-        <v>0.513726</v>
-      </c>
+      <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>0.330391</v>
-      </c>
-      <c r="I34" t="n">
-        <v>0.402149</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I34" t="inlineStr"/>
       <c r="J34" t="n">
-        <v>0.250068</v>
-      </c>
-      <c r="K34" t="n">
-        <v>0.457746</v>
-      </c>
+        <v>0.249811</v>
+      </c>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" t="n">
-        <v>0.347594</v>
-      </c>
-      <c r="M34" t="n">
-        <v>0.395137</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M34" t="inlineStr"/>
       <c r="N34" t="n">
         <v>0.2</v>
       </c>
@@ -3788,7 +3804,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_5.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_19.txt</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
@@ -3818,7 +3834,7 @@
         <v>0.1</v>
       </c>
       <c r="B35" t="n">
-        <v>0.249962</v>
+        <v>0.249907</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -3840,7 +3856,7 @@
       </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="n">
-        <v>0.249766</v>
+        <v>0.249831</v>
       </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="n">
@@ -3881,7 +3897,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_4.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_18.txt</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
@@ -3911,43 +3927,35 @@
         <v>0.1</v>
       </c>
       <c r="B36" t="n">
-        <v>0.234264</v>
+        <v>0.249942</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1790730142</v>
+        <v>1790730194</v>
       </c>
       <c r="E36" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F36" t="n">
         <v>200000</v>
       </c>
-      <c r="G36" t="n">
-        <v>0.626005</v>
-      </c>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>0.588903</v>
-      </c>
-      <c r="I36" t="n">
-        <v>0.606888</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I36" t="inlineStr"/>
       <c r="J36" t="n">
-        <v>0.240798</v>
-      </c>
-      <c r="K36" t="n">
-        <v>0.571429</v>
-      </c>
+        <v>0.249777</v>
+      </c>
+      <c r="K36" t="inlineStr"/>
       <c r="L36" t="n">
-        <v>0.534759</v>
-      </c>
-      <c r="M36" t="n">
-        <v>0.552486</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M36" t="inlineStr"/>
       <c r="N36" t="n">
         <v>0.2</v>
       </c>
@@ -3982,23 +3990,23 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_3.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_1.txt</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z36" t="n">
         <v>12</v>
       </c>
       <c r="AA36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB36" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC36" t="inlineStr">
@@ -4012,43 +4020,35 @@
         <v>0.1</v>
       </c>
       <c r="B37" t="n">
-        <v>0.215814</v>
+        <v>0.249973</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1790730142</v>
+        <v>1790730194</v>
       </c>
       <c r="E37" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F37" t="n">
         <v>200000</v>
       </c>
-      <c r="G37" t="n">
-        <v>0.635251</v>
-      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>0.654477</v>
-      </c>
-      <c r="I37" t="n">
-        <v>0.64472</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="n">
-        <v>0.217291</v>
-      </c>
-      <c r="K37" t="n">
-        <v>0.6282720000000001</v>
-      </c>
+        <v>0.249742</v>
+      </c>
+      <c r="K37" t="inlineStr"/>
       <c r="L37" t="n">
-        <v>0.641711</v>
-      </c>
-      <c r="M37" t="n">
-        <v>0.634921</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M37" t="inlineStr"/>
       <c r="N37" t="n">
         <v>0.2</v>
       </c>
@@ -4083,23 +4083,23 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_11.txt</t>
+          <t>_2_3_3_3_3_1_1790730194_12.txt</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z37" t="n">
         <v>12</v>
       </c>
       <c r="AA37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC37" t="inlineStr">
@@ -4113,7 +4113,7 @@
         <v>0.1</v>
       </c>
       <c r="B38" t="n">
-        <v>0.220684</v>
+        <v>0.22163</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -4130,25 +4130,25 @@
         <v>200000</v>
       </c>
       <c r="G38" t="n">
-        <v>0.590909</v>
+        <v>0.612943</v>
       </c>
       <c r="H38" t="n">
-        <v>0.622951</v>
+        <v>0.633039</v>
       </c>
       <c r="I38" t="n">
-        <v>0.606507</v>
+        <v>0.622829</v>
       </c>
       <c r="J38" t="n">
-        <v>0.221005</v>
+        <v>0.224606</v>
       </c>
       <c r="K38" t="n">
-        <v>0.582915</v>
+        <v>0.596939</v>
       </c>
       <c r="L38" t="n">
-        <v>0.620321</v>
+        <v>0.625668</v>
       </c>
       <c r="M38" t="n">
-        <v>0.601036</v>
+        <v>0.610966</v>
       </c>
       <c r="N38" t="n">
         <v>0.2</v>
@@ -4184,7 +4184,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_8.txt</t>
+          <t>_2_12_1_1790730142_9.txt</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
@@ -4214,42 +4214,42 @@
         <v>0.1</v>
       </c>
       <c r="B39" t="n">
-        <v>0.249509</v>
+        <v>0.215142</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1790730194</v>
+        <v>1790730142</v>
       </c>
       <c r="E39" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F39" t="n">
         <v>200000</v>
       </c>
       <c r="G39" t="n">
-        <v>0.520567</v>
+        <v>0.6676260000000001</v>
       </c>
       <c r="H39" t="n">
-        <v>0.462799</v>
+        <v>0.58512</v>
       </c>
       <c r="I39" t="n">
-        <v>0.489987</v>
+        <v>0.623656</v>
       </c>
       <c r="J39" t="n">
-        <v>0.250785</v>
+        <v>0.215538</v>
       </c>
       <c r="K39" t="n">
-        <v>0.446237</v>
+        <v>0.65896</v>
       </c>
       <c r="L39" t="n">
-        <v>0.44385</v>
+        <v>0.609626</v>
       </c>
       <c r="M39" t="n">
-        <v>0.44504</v>
+        <v>0.633333</v>
       </c>
       <c r="N39" t="n">
         <v>0.2</v>
@@ -4285,23 +4285,23 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790730194_9.txt</t>
+          <t>_2_12_1_1790730142_4.txt</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z39" t="n">
         <v>12</v>
       </c>
       <c r="AA39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC39" t="inlineStr">
@@ -4315,7 +4315,7 @@
         <v>0.1</v>
       </c>
       <c r="B40" t="n">
-        <v>0.211887</v>
+        <v>0.225402</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -4332,25 +4332,25 @@
         <v>200000</v>
       </c>
       <c r="G40" t="n">
-        <v>0.654289</v>
+        <v>0.59611</v>
       </c>
       <c r="H40" t="n">
-        <v>0.644388</v>
+        <v>0.656999</v>
       </c>
       <c r="I40" t="n">
-        <v>0.649301</v>
+        <v>0.625075</v>
       </c>
       <c r="J40" t="n">
-        <v>0.213922</v>
+        <v>0.228309</v>
       </c>
       <c r="K40" t="n">
-        <v>0.644809</v>
+        <v>0.552885</v>
       </c>
       <c r="L40" t="n">
-        <v>0.631016</v>
+        <v>0.614973</v>
       </c>
       <c r="M40" t="n">
-        <v>0.637838</v>
+        <v>0.582278</v>
       </c>
       <c r="N40" t="n">
         <v>0.2</v>
@@ -4386,7 +4386,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_15.txt</t>
+          <t>_2_12_1_1790730142_19.txt</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
@@ -4416,7 +4416,7 @@
         <v>0.1</v>
       </c>
       <c r="B41" t="n">
-        <v>0.22534</v>
+        <v>0.234264</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -4433,25 +4433,25 @@
         <v>200000</v>
       </c>
       <c r="G41" t="n">
-        <v>0.642265</v>
+        <v>0.626005</v>
       </c>
       <c r="H41" t="n">
-        <v>0.586381</v>
+        <v>0.588903</v>
       </c>
       <c r="I41" t="n">
-        <v>0.613052</v>
+        <v>0.606888</v>
       </c>
       <c r="J41" t="n">
-        <v>0.235937</v>
+        <v>0.240798</v>
       </c>
       <c r="K41" t="n">
-        <v>0.559006</v>
+        <v>0.571429</v>
       </c>
       <c r="L41" t="n">
-        <v>0.481283</v>
+        <v>0.534759</v>
       </c>
       <c r="M41" t="n">
-        <v>0.517241</v>
+        <v>0.552486</v>
       </c>
       <c r="N41" t="n">
         <v>0.2</v>
@@ -4487,7 +4487,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>_2_12_1_1790730142_0.txt</t>
+          <t>_2_12_1_1790730142_3.txt</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
@@ -4578,7 +4578,7 @@
         <v>0.6069997</v>
       </c>
       <c r="C2" t="n">
-        <v>0.03963861813420687</v>
+        <v>0.03963861813420686</v>
       </c>
       <c r="D2" t="n">
         <v>0.670051</v>

</xml_diff>